<commit_message>
Auto photo folders: typing a car code creates its Drive folder; photos sync into the sheet
- Photos.gs: per-car folder (shared view-only) with link in photo_folder; syncPhotos fills photos
  (natural file-name order) and auction_sheet_url every 10 min and before Refresh
- Menu: create folders for all cars, sync photos now; drive scope added
- Template, staff guide (BM) and READMEs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DKC2vpBgJkMbEoFZseaZRL
</commit_message>
<xml_diff>
--- a/data/RecondHub-Database.xlsx
+++ b/data/RecondHub-Database.xlsx
@@ -262,12 +262,12 @@
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>Pautan gambar dipisah koma. Gambar pertama = cover.</t>
+        <t>AUTO. Jangan isi. Diisi sendiri dari folder gambar kereta (lajur photo_folder).</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>Pautan gambar auction sheet.</t>
+        <t>AUTO. Diisi sendiri bila ada fail bernama 'auction' dalam folder gambar.</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
@@ -293,6 +293,11 @@
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>Tarikh terjual (auto diisi bila status = Sold).</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>AUTO. Pautan folder gambar kereta ini. Klik dan drag gambar masuk. Gambar 01 = gambar utama.</t>
       </text>
     </comment>
   </commentList>
@@ -945,7 +950,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Muat naik ke Google Drive, Share &gt; Anyone with the link &gt; Viewer, copy link. Tampal dalam photos dipisah koma. Gambar pertama = gambar utama.</t>
+          <t>Taip kod kereta dahulu. Folder gambar akan dibuat sendiri dan pautannya muncul dalam lajur photo_folder. Klik pautan, drag gambar masuk, namakan 01, 02, 03 (01 = gambar utama). Auction sheet: namakan fail 'auction'. Lajur photos diisi sendiri setiap 10 minit atau bila tekan Refresh website.</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1068,13 +1073,14 @@
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="15" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
     <col width="28" customWidth="1" min="19" max="19"/>
     <col width="38" customWidth="1" min="20" max="20"/>
     <col width="45" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1198,6 +1204,11 @@
           <t>sold_date</t>
         </is>
       </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>photo_folder</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -1308,6 +1319,7 @@
         </is>
       </c>
       <c r="X2" s="6" t="inlineStr"/>
+      <c r="Y2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -1418,6 +1430,7 @@
         </is>
       </c>
       <c r="X3" s="6" t="inlineStr"/>
+      <c r="Y3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1532,6 +1545,7 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="Y4" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="7">

</xml_diff>

<commit_message>
Clarify 'auction sheet' = Japanese inspection report (site labels, staff guide, sheet template)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DKC2vpBgJkMbEoFZseaZRL
</commit_message>
<xml_diff>
--- a/data/RecondHub-Database.xlsx
+++ b/data/RecondHub-Database.xlsx
@@ -227,7 +227,7 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Gred lelongan, cth. 4.5</t>
+        <t>Gred dari auction sheet (laporan pemeriksaan Jepun), cth. 4.5</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -267,7 +267,7 @@
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>AUTO. Diisi sendiri bila ada fail bernama 'auction' dalam folder gambar.</t>
+        <t>AUTO. Auction sheet = laporan pemeriksaan kereta dari Jepun (gred, mileage, calar). BUKAN lelongan. Diisi sendiri bila ada fail bernama 'auction' dalam folder gambar kereta.</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
@@ -823,7 +823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Taip kod kereta dahulu. Folder gambar akan dibuat sendiri dan pautannya muncul dalam lajur photo_folder. Klik pautan, drag gambar masuk, namakan 01, 02, 03 (01 = gambar utama). Auction sheet: namakan fail 'auction'. Lajur photos diisi sendiri setiap 10 minit atau bila tekan Refresh website.</t>
+          <t>Taip kod kereta dahulu. Folder gambar akan dibuat sendiri dan pautannya muncul dalam lajur photo_folder. Klik pautan, drag gambar masuk, namakan 01, 02, 03 (01 = gambar utama). Auction sheet (laporan pemeriksaan dari Jepun, bukan lelongan): ambil gambar dokumen itu dan namakan fail 'auction'. Lajur photos diisi sendiri setiap 10 minit atau bila tekan Refresh website.</t>
         </is>
       </c>
     </row>
@@ -997,46 +997,58 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Tab Showrooms</t>
+          <t>Auction sheet?</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Satu baris = satu showroom. opening_hours cth: Mon-Sat 10:00-19:00; Sun 11:00-17:00 (slot tempahan dijana dari sini).</t>
+          <t>Laporan pemeriksaan yang ditulis di Jepun semasa kereta dibeli (gred, mileage, peta calar). Ia BUKAN lelongan oleh syarikat. Satu kereta = satu dokumen, letak gambarnya dalam folder gambar kereta yang sama.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Tab Agents</t>
+          <t>Tab Showrooms</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Satu baris = satu agen. state = negeri, atau HQ untuk sales advisor HQ. active FALSE = berhenti terima lead.</t>
+          <t>Satu baris = satu showroom. opening_hours cth: Mon-Sat 10:00-19:00; Sun 11:00-17:00 (slot tempahan dijana dari sini).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Tab Settings</t>
+          <t>Tab Agents</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Satu baris sahaja: nombor WhatsApp HQ &amp; owner, kadar faedah lalai, tempoh maksimum, deposit minimum.</t>
+          <t>Satu baris = satu agen. state = negeri, atau HQ untuk sales advisor HQ. active FALSE = berhenti terima lead.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Tab Settings</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Satu baris sahaja: nombor WhatsApp HQ &amp; owner, kadar faedah lalai, tempoh maksimum, deposit minimum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Tab Leads</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Diisi oleh laman web. Jangan taip di sini kecuali menukar lajur status (cth. Contacted, Booked, Sold, Lost).</t>
         </is>

</xml_diff>

<commit_message>
Friendly BM sheet columns, car features and seats
- Sheet headers can be BM labels (Kod Kereta, Harga (RM)…) or internal keys; one mapping in columns.ts
  (mirrored in Apps Script Config.gs)
- New stock data: seats, drivetrain, 12 feature tick-boxes (sunroof, pilot seat, power doors…)
- Website: features list on car pages, seats in cards/specs, feature and seat filters, features searchable
- Leads written in plain BM (Jenis: Tempah Tontonan…, readable Maklumat Tambahan)
- Client template regenerated; staff guide and README updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DKC2vpBgJkMbEoFZseaZRL
</commit_message>
<xml_diff>
--- a/data/RecondHub-Database.xlsx
+++ b/data/RecondHub-Database.xlsx
@@ -44,7 +44,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000E1116"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F7A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B7280"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,12 +97,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -167,371 +183,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RecondHub</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Kod unik kereta, cth. RH121. Jangan guna semula kod lama.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Available / Reserved / Sold / Hidden</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Jenama, cth. Toyota</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Model, cth. Alphard. Eja sama setiap kali.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Varian, cth. 2.5 SC</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Tahun dibuat, cth. 2021</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Tahun daftar. Kosongkan jika belum daftar.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. MPV / SUV / Sedan / Hatchback / Coupe / Pickup</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Harga dalam RM, nombor sahaja, cth. 238000</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Mileage dalam km, cth. 32000</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Gred dari auction sheet (laporan pemeriksaan Jepun), cth. 4.5</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>Kapasiti enjin cc, cth. 2494</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Automatic / Manual</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>Petrol / Hybrid / Diesel / Plug-in Hybrid / Electric</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Warna, cth. Pearl White</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>Pilih dari tab Showrooms. Kosongkan untuk kereta AP rakan (isi state).</t>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <t>Wajib jika tiada showroom_id.</t>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <t>AUTO. Jangan isi. Diisi sendiri dari folder gambar kereta (lajur photo_folder).</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>AUTO. Auction sheet = laporan pemeriksaan kereta dari Jepun (gred, mileage, calar). BUKAN lelongan. Diisi sendiri bila ada fail bernama 'auction' dalam folder gambar kereta.</t>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <t>Kelebihan dipisah koma, cth. Pilot seats, Sunroof, JBL</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>Penerangan ringkas kereta.</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>TRUE = dipapar di halaman utama</t>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <t>Tarikh masuk stok, cth. 2026-10-02 (auto diisi oleh Apps Script).</t>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <t>Tarikh terjual (auto diisi bila status = Sold).</t>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <t>AUTO. Pautan folder gambar kereta ini. Klik dan drag gambar masuk. Gambar 01 = gambar utama.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RecondHub</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Kod unik, cth. SR01</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Nama showroom, cth. RecondHub HQ Shah Alam</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Negeri</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Bandar</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Alamat penuh</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Pautan Google Maps</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. WhatsApp showroom, format 60XXXXXXXXX</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>cth. Mon-Sat 10:00-19:00; Sun 11:00-17:00</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Pautan gambar showroom</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RecondHub</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Kod unik, cth. A01 (agen negeri) atau H01 (SA HQ). Jangan tukar selepas digunakan.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Nama penuh</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Negeri liputan, atau HQ untuk sales advisor HQ</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Showroom asal (pilihan)</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Format 60XXXXXXXXX</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Pautan gambar muka (pilihan)</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. TRUE = terima lead, FALSE = berhenti</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RecondHub</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. WhatsApp HQ (fallback untuk semua lead)</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. WhatsApp owner untuk Private Sourcing sahaja</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Kadar faedah lalai kalkulator, % flat setahun, cth. 3.0</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Tempoh maksimum pinjaman (tahun), cth. 9</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>WAJIB. Deposit minimum %, cth. 10</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>DSR di bawah nilai ini = Likely eligible (lalai 60)</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>DSR sehingga nilai ini = Borderline (lalai 70)</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>RecondHub</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Diisi oleh laman web</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Jenis lead</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Maklumat tambahan</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Agen/showroom yang menerima lead</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t/>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>New bila masuk. Staf tukar ke Contacted / Booked / Test drive / Loan submitted / Sold / Lost</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -823,17 +474,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RecondHub: Database Laman Web</t>
+          <t>RecondHub: Database Website</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -850,207 +501,219 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Isi tab Stock, Showrooms, Agents dan Settings. Laman web membaca sheet ini secara automatik (setiap 5 minit).</t>
+          <t>Isi tab Stock, Showrooms, Agents dan Settings. Website membaca sheet ini sendiri setiap 5 minit.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Baris kelabu</t>
+          <t>Warna header</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Baris kelabu di setiap tab ialah CONTOH. Gantikan atau padam sebelum laman dilancarkan.</t>
+          <t>EMAS = wajib diisi · HITAM = pilihan · HIJAU = ciri kereta (pilih TRUE kalau ada) · KELABU = automatik, jangan isi.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Lajur emas</t>
+          <t>Baris kelabu muda</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Header berwarna emas = WAJIB diisi. Header hitam = pilihan.</t>
+          <t>Contoh sahaja. Gantikan atau padam sebelum website dilancarkan.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Nota lajur</t>
+          <t>Senarai pilihan</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Letak tetikus atas header untuk lihat penerangan setiap lajur.</t>
+          <t>Lajur seperti Status, Jenis Badan, Negeri dan Showroom ada senarai pilihan. Pilih dari senarai.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Dropdown</t>
+          <t>Jangan ubah</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Lajur seperti status, body_type, state dan showroom_id ada senarai pilihan. Sila pilih dari senarai.</t>
+          <t>Jangan tukar nama tab atau nama lajur di baris 1. Jangan padam tab Lists dan Leads.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Jangan ubah</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Jangan tukar nama tab atau nama header di baris 1. Jangan padam tab Lists dan Leads.</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TAB STOCK</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Satu baris = satu kereta. Kod Kereta mesti unik (cth. RH121). Kereta terjual: tukar Status ke Sold (jangan padam baris).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Tab Stock</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Satu baris = satu kereta. code mesti unik (cth. RH121). Untuk kereta terjual, tukar status ke Sold (jangan padam baris).</t>
+          <t>Available = dijual · Reserved = ditempah · Sold = terjual (dipapar 7 hari dengan tanda Sold) · Hidden = tidak dipapar.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Ciri kereta (hijau)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Available = dijual · Reserved = ditempah (masih dipapar) · Sold = terjual (dipapar 7 hari dengan lencana Sold) · Hidden = tidak dipapar.</t>
+          <t>Pilih TRUE untuk setiap ciri yang ada (Sunroof, Pilot Seat dan lain-lain). Biarkan kosong kalau tiada. Pelanggan boleh tapis kereta ikut ciri ini.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Gambar</t>
+          <t>Kelebihan Lain</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Taip kod kereta dahulu. Folder gambar akan dibuat sendiri dan pautannya muncul dalam lajur photo_folder. Klik pautan, drag gambar masuk, namakan 01, 02, 03 (01 = gambar utama). Auction sheet (laporan pemeriksaan dari Jepun, bukan lelongan): ambil gambar dokumen itu dan namakan fail 'auction'. Lajur photos diisi sendiri setiap 10 minit atau bila tekan Refresh website.</t>
+          <t>Ciri lain yang tiada dalam senarai, dipisah koma. Cth: Modellista bodykit, JBL, Digital mirror.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Harga &amp; nombor</t>
+          <t>Gambar</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Tulis nombor sahaja (238000). RM dan koma pun diterima.</t>
+          <t>Taip Kod Kereta dahulu. Folder gambar dibuat sendiri dan pautannya muncul dalam lajur Folder Gambar. Klik, masukkan gambar, namakan 01, 02, 03 (01 = gambar utama).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Tarikh</t>
+          <t>Auction sheet</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Format 2026-10-02 atau 02/10/2026.</t>
+          <t>Laporan pemeriksaan dari Jepun semasa kereta dibeli (gred, mileage, calar). BUKAN lelongan. Ambil gambar dokumen itu, masukkan dalam folder gambar kereta, namakan fail 'auction'.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Harga &amp; nombor</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Format 60123456789 (tanpa +, tanpa sengkang).</t>
+          <t>Tulis nombor sahaja (238000). RM dan koma pun diterima.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Tarikh</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Format 2026-10-02 atau 02/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Auction sheet?</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Laporan pemeriksaan yang ditulis di Jepun semasa kereta dibeli (gred, mileage, peta calar). Ia BUKAN lelongan oleh syarikat. Satu kereta = satu dokumen, letak gambarnya dalam folder gambar kereta yang sama.</t>
+          <t>Format 60123456789 (tanpa +, tanpa sengkang).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Tab Showrooms</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Satu baris = satu showroom. opening_hours cth: Mon-Sat 10:00-19:00; Sun 11:00-17:00 (slot tempahan dijana dari sini).</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Tab Agents</t>
+          <t>TAB SHOWROOMS</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Satu baris = satu agen. state = negeri, atau HQ untuk sales advisor HQ. active FALSE = berhenti terima lead.</t>
+          <t>Satu baris = satu showroom. Waktu Operasi cth: Mon-Sat 10:00-19:00; Sun 11:00-17:00 (slot tempahan dijana dari sini).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Tab Settings</t>
+          <t>TAB AGENTS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Satu baris sahaja: nombor WhatsApp HQ &amp; owner, kadar faedah lalai, tempoh maksimum, deposit minimum.</t>
+          <t>Satu baris = satu agen. Negeri = kawasan agen, atau HQ untuk sales advisor HQ. Aktif FALSE = berhenti terima pelanggan.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Tab Leads</t>
+          <t>TAB SETTINGS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Diisi oleh laman web. Jangan taip di sini kecuali menukar lajur status (cth. Contacted, Booked, Sold, Lost).</t>
+          <t>Satu baris sahaja: nombor WhatsApp HQ &amp; owner, kadar faedah, tempoh dan deposit minimum untuk kalkulator pinjaman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TAB LEADS</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Diisi oleh website setiap kali pelanggan hubungi. Staf hanya tukar lajur Status (Contacted, Booked, Sold, Lost).</t>
         </is>
       </c>
     </row>
@@ -1065,526 +728,722 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:AM4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="28" customWidth="1" min="19" max="19"/>
-    <col width="38" customWidth="1" min="20" max="20"/>
-    <col width="45" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="31" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="34" customWidth="1" min="30" max="30"/>
+    <col width="40" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="24" customWidth="1" min="34" max="34"/>
+    <col width="34" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="23" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="38" max="38"/>
+    <col width="14" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>Kod Kereta</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>make</t>
+          <t>Jenama</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>variant</t>
+          <t>Varian</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>year_manufactured</t>
+          <t>Tahun Dibuat</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>year_registered</t>
+          <t>Tahun Daftar</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>body_type</t>
+          <t>Jenis Badan</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>price_rm</t>
+          <t>Harga (RM)</t>
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
-          <t>mileage_km</t>
+          <t>Mileage (km)</t>
         </is>
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
-          <t>grade</t>
+          <t>Gred Auction</t>
         </is>
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>engine_cc</t>
+          <t>Enjin (cc)</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
         <is>
-          <t>transmission</t>
+          <t>Gear</t>
         </is>
       </c>
       <c r="N1" s="5" t="inlineStr">
         <is>
-          <t>fuel</t>
+          <t>Minyak</t>
         </is>
       </c>
       <c r="O1" s="5" t="inlineStr">
         <is>
-          <t>colour</t>
+          <t>Warna</t>
         </is>
       </c>
       <c r="P1" s="5" t="inlineStr">
         <is>
-          <t>showroom_id</t>
+          <t>Tempat Duduk</t>
         </is>
       </c>
       <c r="Q1" s="5" t="inlineStr">
         <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="R1" s="5" t="inlineStr">
-        <is>
-          <t>photos</t>
-        </is>
-      </c>
-      <c r="S1" s="5" t="inlineStr">
-        <is>
-          <t>auction_sheet_url</t>
-        </is>
-      </c>
-      <c r="T1" s="5" t="inlineStr">
-        <is>
-          <t>highlights</t>
-        </is>
-      </c>
-      <c r="U1" s="5" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="V1" s="5" t="inlineStr">
-        <is>
-          <t>featured</t>
-        </is>
-      </c>
-      <c r="W1" s="5" t="inlineStr">
-        <is>
-          <t>date_added</t>
-        </is>
-      </c>
-      <c r="X1" s="5" t="inlineStr">
-        <is>
-          <t>sold_date</t>
-        </is>
-      </c>
-      <c r="Y1" s="5" t="inlineStr">
-        <is>
-          <t>photo_folder</t>
+          <t>Pacuan</t>
+        </is>
+      </c>
+      <c r="R1" s="6" t="inlineStr">
+        <is>
+          <t>Sunroof</t>
+        </is>
+      </c>
+      <c r="S1" s="6" t="inlineStr">
+        <is>
+          <t>Moonroof / Panoramic</t>
+        </is>
+      </c>
+      <c r="T1" s="6" t="inlineStr">
+        <is>
+          <t>Pintu Elektrik</t>
+        </is>
+      </c>
+      <c r="U1" s="6" t="inlineStr">
+        <is>
+          <t>Bonet Elektrik</t>
+        </is>
+      </c>
+      <c r="V1" s="6" t="inlineStr">
+        <is>
+          <t>Pilot Seat</t>
+        </is>
+      </c>
+      <c r="W1" s="6" t="inlineStr">
+        <is>
+          <t>Kerusi Kulit</t>
+        </is>
+      </c>
+      <c r="X1" s="6" t="inlineStr">
+        <is>
+          <t>Kamera 360</t>
+        </is>
+      </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>Skrin Belakang</t>
+        </is>
+      </c>
+      <c r="Z1" s="6" t="inlineStr">
+        <is>
+          <t>Head-Up Display</t>
+        </is>
+      </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
+          <t>Audio Premium</t>
+        </is>
+      </c>
+      <c r="AB1" s="6" t="inlineStr">
+        <is>
+          <t>Apple CarPlay / Android Auto</t>
+        </is>
+      </c>
+      <c r="AC1" s="6" t="inlineStr">
+        <is>
+          <t>Adaptive Cruise</t>
+        </is>
+      </c>
+      <c r="AD1" s="5" t="inlineStr">
+        <is>
+          <t>Kelebihan Lain</t>
+        </is>
+      </c>
+      <c r="AE1" s="5" t="inlineStr">
+        <is>
+          <t>Penerangan</t>
+        </is>
+      </c>
+      <c r="AF1" s="5" t="inlineStr">
+        <is>
+          <t>Showroom</t>
+        </is>
+      </c>
+      <c r="AG1" s="5" t="inlineStr">
+        <is>
+          <t>Negeri</t>
+        </is>
+      </c>
+      <c r="AH1" s="5" t="inlineStr">
+        <is>
+          <t>Tonjol di Laman Utama</t>
+        </is>
+      </c>
+      <c r="AI1" s="7" t="inlineStr">
+        <is>
+          <t>Folder Gambar</t>
+        </is>
+      </c>
+      <c r="AJ1" s="7" t="inlineStr">
+        <is>
+          <t>Gambar (auto)</t>
+        </is>
+      </c>
+      <c r="AK1" s="7" t="inlineStr">
+        <is>
+          <t>Auction Sheet (auto)</t>
+        </is>
+      </c>
+      <c r="AL1" s="7" t="inlineStr">
+        <is>
+          <t>Tarikh Masuk</t>
+        </is>
+      </c>
+      <c r="AM1" s="7" t="inlineStr">
+        <is>
+          <t>Tarikh Jual</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>RH101</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Alphard</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>2.5 SC</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>MPV</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>238000</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>32000</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t>2494</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Automatic</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="N2" s="8" t="inlineStr">
         <is>
           <t>Petrol</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O2" s="8" t="inlineStr">
         <is>
           <t>Pearl White</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="P2" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>2WD</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="U2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="V2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AA2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC2" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD2" s="8" t="inlineStr">
+        <is>
+          <t>Digital inner mirror, Modellista bodykit</t>
+        </is>
+      </c>
+      <c r="AE2" s="8" t="inlineStr">
+        <is>
+          <t>Clean SC with pilot seats and sunroof. Auction grade 4.5.</t>
+        </is>
+      </c>
+      <c r="AF2" s="8" t="inlineStr">
         <is>
           <t>SR01</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="AG2" s="8" t="inlineStr">
         <is>
           <t>Selangor</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr"/>
-      <c r="S2" s="6" t="inlineStr"/>
-      <c r="T2" s="6" t="inlineStr">
-        <is>
-          <t>Pilot seats, Power boot, Sunroof, JBL sound</t>
-        </is>
-      </c>
-      <c r="U2" s="6" t="inlineStr">
-        <is>
-          <t>Clean SC with pilot seats and sunroof. Auction grade 4.5.</t>
-        </is>
-      </c>
-      <c r="V2" s="6" t="inlineStr">
+      <c r="AH2" s="8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="W2" s="6" t="inlineStr">
+      <c r="AL2" s="8" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="X2" s="6" t="inlineStr"/>
-      <c r="Y2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>RH102</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Reserved</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Harrier</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>2.0 Z Leather</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>SUV</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>199000</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>25000</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>1986</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Automatic</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Petrol</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Precious Black Pearl</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>2WD</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="U3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AA3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AC3" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AE3" s="8" t="inlineStr">
+        <is>
+          <t>Harrier Z Leather dengan panoramic roof.</t>
+        </is>
+      </c>
+      <c r="AF3" s="8" t="inlineStr">
         <is>
           <t>SR02</t>
         </is>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="AG3" s="8" t="inlineStr">
         <is>
           <t>Johor</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr"/>
-      <c r="S3" s="6" t="inlineStr"/>
-      <c r="T3" s="6" t="inlineStr">
-        <is>
-          <t>Leather package, Panoramic roof</t>
-        </is>
-      </c>
-      <c r="U3" s="6" t="inlineStr">
-        <is>
-          <t>Harrier Z Leather dengan panoramic roof.</t>
-        </is>
-      </c>
-      <c r="V3" s="6" t="inlineStr">
+      <c r="AH3" s="8" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="W3" s="6" t="inlineStr">
+      <c r="AL3" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="X3" s="6" t="inlineStr"/>
-      <c r="Y3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>RH103</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Sold</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Honda</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Civic</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Type R FK8</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Hatchback</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>318000</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>22000</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>1996</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Petrol</t>
         </is>
       </c>
-      <c r="O4" s="6" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>Championship White</t>
         </is>
       </c>
-      <c r="P4" s="6" t="inlineStr">
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>2WD</t>
+        </is>
+      </c>
+      <c r="AB4" s="8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AD4" s="8" t="inlineStr">
+        <is>
+          <t>6-speed manual, Brembo brakes, Recaro seats</t>
+        </is>
+      </c>
+      <c r="AE4" s="8" t="inlineStr">
+        <is>
+          <t>Unmodified FK8 Type R.</t>
+        </is>
+      </c>
+      <c r="AF4" s="8" t="inlineStr">
         <is>
           <t>SR01</t>
         </is>
       </c>
-      <c r="Q4" s="6" t="inlineStr">
+      <c r="AG4" s="8" t="inlineStr">
         <is>
           <t>Selangor</t>
         </is>
       </c>
-      <c r="R4" s="6" t="inlineStr"/>
-      <c r="S4" s="6" t="inlineStr"/>
-      <c r="T4" s="6" t="inlineStr">
-        <is>
-          <t>6-speed manual, Brembo brakes</t>
-        </is>
-      </c>
-      <c r="U4" s="6" t="inlineStr">
-        <is>
-          <t>Unmodified FK8 Type R.</t>
-        </is>
-      </c>
-      <c r="V4" s="6" t="inlineStr">
+      <c r="AH4" s="8" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="W4" s="6" t="inlineStr">
+      <c r="AL4" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="X4" s="6" t="inlineStr">
+      <c r="AM4" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="Y4" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Available / Reserved / Sold / Hidden" type="list">
+  <dataValidations count="20">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"Available,Reserved,Sold,Hidden"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Jenis badan" type="list">
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"MPV,SUV,Sedan,Hatchback,Coupe,Pickup"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Transmisi" type="list">
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"Automatic,Manual"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Bahan api" type="list">
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"Petrol,Hybrid,Diesel,Plug-in Hybrid,Electric"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Pilih showroom_id" type="list">
+    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"2WD,4WD,AWD"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF2:AF500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>Showrooms!$A$2:$A$200</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Pilih negeri" type="list">
+    <dataValidation sqref="AG2:AG500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>Lists!$A$2:$A$17</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="TRUE = featured" type="list">
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA2:AA500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2:AB500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AH2:AH500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1598,157 +1457,154 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>showroom_id</t>
+          <t>Kod Showroom</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Nama</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>Negeri</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>Bandar</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>Alamat</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>google_maps_url</t>
+          <t>Pautan Google Maps</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>opening_hours</t>
+          <t>Waktu Operasi</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>Gambar</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>SR01</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>RecondHub HQ Shah Alam</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Selangor</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Shah Alam</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Lot 12, Jalan Contoh, Seksyen 15, 40200 Shah Alam</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>https://maps.google.com/?q=Shah+Alam</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>60123456701</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Mon-Sat 10:00-19:00; Sun 11:00-17:00</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>SR02</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>RecondHub Johor Bahru</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Johor</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Johor Bahru</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>No. 8, Jalan Contoh, 81100 Johor Bahru</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>https://maps.google.com/?q=Johor+Bahru</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>60123456702</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Daily 10:00-19:00</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Pilih negeri" type="list">
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>Lists!$A$2:$A$17</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1761,113 +1617,111 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>agent_id</t>
+          <t>Kod Agen</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Nama</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>Negeri</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>showroom_id</t>
+          <t>Showroom</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>Gambar</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Aktif</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Nama Agen Johor</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Johor</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>SR02</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>60133333301</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Nama SA HQ</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>HQ</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>SR01</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>60133333311</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1875,18 +1729,17 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Negeri atau HQ" type="list">
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>Lists!$B$2:$B$18</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Pilih showroom_id" type="list">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>Showrooms!$A$2:$A$200</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Aktif?" type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1899,84 +1752,84 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>hq_whatsapp</t>
+          <t>WhatsApp HQ</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>owner_whatsapp</t>
+          <t>WhatsApp Owner</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>default_interest_rate</t>
+          <t>Kadar Faedah (%)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>max_tenure_years</t>
+          <t>Tempoh Maksimum (tahun)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>min_downpayment_pct</t>
+          <t>Deposit Minimum (%)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>dsr_eligible_max</t>
+          <t>Had Layak Pinjaman (%)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>dsr_borderline_max</t>
+          <t>Had Sempadan Pinjaman (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>60123456700</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>60129999999</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>70</t>
         </is>
@@ -1984,7 +1837,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1997,108 +1849,107 @@
   <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>Masa</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>Jenis</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>car_code</t>
+          <t>Kod Kereta</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Nama</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>Telefon</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>Negeri</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>showroom_id</t>
+          <t>Showroom</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>preferred_date</t>
+          <t>Tarikh Pilihan</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>preferred_time</t>
+          <t>Masa Pilihan</t>
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
-          <t>details_json</t>
+          <t>Maklumat Tambahan</t>
         </is>
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
-          <t>assigned_to</t>
+          <t>Diserah Kepada</t>
         </is>
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>source_page</t>
+          <t>Halaman</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
         <is>
-          <t>utm_source</t>
+          <t>Sumber Iklan</t>
         </is>
       </c>
       <c r="N1" s="5" t="inlineStr">
         <is>
-          <t>utm_campaign</t>
+          <t>Kempen Iklan</t>
         </is>
       </c>
       <c r="O1" s="5" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak sah" error="Sila pilih dari senarai." promptTitle="Pilih" prompt="Status lead" type="list">
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tidak sah" error="Sila pilih dari senarai." type="list">
       <formula1>"New,Contacted,Booked,Test drive,Loan submitted,Sold,Lost"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2114,12 +1965,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>states</t>
+          <t>Negeri</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>states_hq</t>
+          <t>Negeri + HQ</t>
         </is>
       </c>
     </row>

</xml_diff>